<commit_message>
data: actualitzar tasca 02.20 — llistats, referència i metadades
Actualització dels llistats xlsx de l'alumne 5796, referencia.json
i config.json de la tasca 02.20/ADG32.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/tasques/02.20/ADG32/entregues/5796/02.20-5796-02_RECEPCIONS.xlsx
+++ b/data/tasques/02.20/ADG32/entregues/5796/02.20-5796-02_RECEPCIONS.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="120">
   <si>
     <t>Referencia</t>
   </si>
@@ -43,7 +43,7 @@
     <t>MGZ01/ENTRA/00001</t>
   </si>
   <si>
-    <t>00004</t>
+    <t>00005</t>
   </si>
   <si>
     <t>ROCALLA SA</t>
@@ -58,7 +58,7 @@
     <t>MGZ01/ENTRA/00002</t>
   </si>
   <si>
-    <t>00003</t>
+    <t>00001</t>
   </si>
   <si>
     <t>ALUBIX SL</t>
@@ -70,7 +70,7 @@
     <t>MGZ01/ENTRA/00003</t>
   </si>
   <si>
-    <t>00008</t>
+    <t>00010</t>
   </si>
   <si>
     <t>C-C/00003</t>
@@ -79,157 +79,154 @@
     <t>MGZ01/ENTRA/00004</t>
   </si>
   <si>
-    <t>00006</t>
+    <t>MGZ01/ENTRA/00005</t>
   </si>
   <si>
     <t>C-C/00004</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00005</t>
-  </si>
-  <si>
-    <t>00010</t>
+    <t>MGZ01/ENTRA/00007</t>
+  </si>
+  <si>
+    <t>00013</t>
   </si>
   <si>
     <t>C-C/00005</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00006</t>
+    <t>MGZ01/ENTRA/00008</t>
+  </si>
+  <si>
+    <t>00015</t>
   </si>
   <si>
     <t>C-C/00006</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00007</t>
-  </si>
-  <si>
-    <t>00011</t>
+    <t>MGZ01/ENTRA/00009</t>
+  </si>
+  <si>
+    <t>00017</t>
   </si>
   <si>
     <t>C-C/00007</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00008</t>
-  </si>
-  <si>
-    <t>00012</t>
+    <t>MGZ01/ENTRA/00010</t>
   </si>
   <si>
     <t>C-C/00008</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00009</t>
-  </si>
-  <si>
-    <t>00015</t>
+    <t>MGZ01/ENTRA/00011</t>
+  </si>
+  <si>
+    <t>00018</t>
   </si>
   <si>
     <t>C-C/00009</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00010</t>
+    <t>MGZ01/ENTRA/00012</t>
+  </si>
+  <si>
+    <t>00020</t>
   </si>
   <si>
     <t>C-C/00010</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00011</t>
-  </si>
-  <si>
-    <t>00020</t>
+    <t>MGZ01/ENTRA/00013</t>
+  </si>
+  <si>
+    <t>00022</t>
   </si>
   <si>
     <t>C-C/00011</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00012</t>
-  </si>
-  <si>
-    <t>00019</t>
+    <t>MGZ01/ENTRA/00014</t>
   </si>
   <si>
     <t>C-C/00012</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00013</t>
-  </si>
-  <si>
-    <t>00021</t>
+    <t>MGZ01/ENTRA/00015</t>
+  </si>
+  <si>
+    <t>00027</t>
   </si>
   <si>
     <t>C-C/00013</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00014</t>
+    <t>MGZ01/ENTRA/00016</t>
+  </si>
+  <si>
+    <t>00023</t>
   </si>
   <si>
     <t>C-C/00014</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00015</t>
-  </si>
-  <si>
-    <t>00025</t>
+    <t>MGZ01/ENTRA/00018</t>
+  </si>
+  <si>
+    <t>00031</t>
   </si>
   <si>
     <t>C-C/00015</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00016</t>
-  </si>
-  <si>
-    <t>00024</t>
+    <t>MGZ01/ENTRA/00019</t>
   </si>
   <si>
     <t>C-C/00016</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00017</t>
-  </si>
-  <si>
-    <t>00029</t>
+    <t>MGZ01/ENTRA/00020</t>
+  </si>
+  <si>
+    <t>00030</t>
   </si>
   <si>
     <t>C-C/00017</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00018</t>
-  </si>
-  <si>
-    <t>00026</t>
+    <t>MGZ01/ENTRA/00022</t>
+  </si>
+  <si>
+    <t>00032</t>
   </si>
   <si>
     <t>C-C/00018</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00019</t>
-  </si>
-  <si>
-    <t>00032</t>
+    <t>MGZ01/ENTRA/00023</t>
   </si>
   <si>
     <t>C-C/00019</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00020</t>
-  </si>
-  <si>
-    <t>00031</t>
+    <t>MGZ01/ENTRA/00024</t>
+  </si>
+  <si>
+    <t>00033</t>
   </si>
   <si>
     <t>C-C/00020</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00021</t>
-  </si>
-  <si>
-    <t>00036</t>
+    <t>MGZ01/ENTRA/00025</t>
+  </si>
+  <si>
+    <t>00035</t>
   </si>
   <si>
     <t>C-C/00021</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00022</t>
+    <t>MGZ01/ENTRA/00026</t>
   </si>
   <si>
     <t>00034</t>
@@ -238,106 +235,145 @@
     <t>C-C/00022</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00023</t>
-  </si>
-  <si>
-    <t>00037</t>
+    <t>MGZ01/ENTRA/00027</t>
+  </si>
+  <si>
+    <t>00039</t>
   </si>
   <si>
     <t>C-C/00023</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00024</t>
-  </si>
-  <si>
-    <t>00035</t>
+    <t>MGZ01/ENTRA/00028</t>
+  </si>
+  <si>
+    <t>00038</t>
   </si>
   <si>
     <t>C-C/00024</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00025</t>
+    <t>MGZ01/ENTRA/00029</t>
+  </si>
+  <si>
+    <t>00040</t>
+  </si>
+  <si>
+    <t>C-C/00025</t>
+  </si>
+  <si>
+    <t>MGZ01/ENTRA/00030</t>
   </si>
   <si>
     <t>00041</t>
   </si>
   <si>
-    <t>C-C/00025</t>
-  </si>
-  <si>
-    <t>MGZ01/ENTRA/00026</t>
-  </si>
-  <si>
-    <t>00039</t>
-  </si>
-  <si>
     <t>C-C/00026</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00027</t>
+    <t>MGZ01/ENTRA/00031</t>
+  </si>
+  <si>
+    <t>00043</t>
+  </si>
+  <si>
+    <t>C-C/00027</t>
+  </si>
+  <si>
+    <t>MGZ01/ENTRA/00032</t>
+  </si>
+  <si>
+    <t>00044</t>
+  </si>
+  <si>
+    <t>C-C/00028</t>
+  </si>
+  <si>
+    <t>MGZ01/ENTRA/00033</t>
   </si>
   <si>
     <t>00046</t>
   </si>
   <si>
-    <t>C-C/00027</t>
-  </si>
-  <si>
-    <t>MGZ01/ENTRA/00028</t>
-  </si>
-  <si>
-    <t>C-C/00028</t>
-  </si>
-  <si>
-    <t>MGZ01/ENTRA/00029</t>
-  </si>
-  <si>
-    <t>00050</t>
-  </si>
-  <si>
     <t>C-C/00029</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00030</t>
-  </si>
-  <si>
-    <t>00045</t>
+    <t>MGZ01/ENTRA/00034</t>
+  </si>
+  <si>
+    <t>00049</t>
   </si>
   <si>
     <t>C-C/00030</t>
   </si>
   <si>
-    <t>MGZ01/ENTRA/00031</t>
+    <t>MGZ01/ENTRA/00035</t>
+  </si>
+  <si>
+    <t>00048</t>
+  </si>
+  <si>
+    <t>C-C/00031</t>
+  </si>
+  <si>
+    <t>MGZ01/ENTRA/00036</t>
+  </si>
+  <si>
+    <t>00051</t>
+  </si>
+  <si>
+    <t>C-C/00032</t>
+  </si>
+  <si>
+    <t>MGZ01/ENTRA/00037</t>
   </si>
   <si>
     <t>00052</t>
   </si>
   <si>
-    <t>C-C/00031</t>
-  </si>
-  <si>
-    <t>MGZ01/ENTRA/00032</t>
-  </si>
-  <si>
-    <t>00049</t>
-  </si>
-  <si>
-    <t>C-C/00032</t>
-  </si>
-  <si>
-    <t>MGZ01/ENTRA/00033</t>
+    <t>C-C/00033</t>
+  </si>
+  <si>
+    <t>MGZ01/ENTRA/00038</t>
   </si>
   <si>
     <t>00053</t>
   </si>
   <si>
-    <t>C-C/00033</t>
-  </si>
-  <si>
-    <t>MGZ01/ENTRA/00034</t>
-  </si>
-  <si>
     <t>C-C/00034</t>
+  </si>
+  <si>
+    <t>MGZ01/ENTRA/00039</t>
+  </si>
+  <si>
+    <t>00058</t>
+  </si>
+  <si>
+    <t>C-C/00035</t>
+  </si>
+  <si>
+    <t>MGZ01/ENTRA/00040</t>
+  </si>
+  <si>
+    <t>C-C/00036</t>
+  </si>
+  <si>
+    <t>MGZ01/ENTRA/00041</t>
+  </si>
+  <si>
+    <t>00055</t>
+  </si>
+  <si>
+    <t>C-C/00037</t>
+  </si>
+  <si>
+    <t>MGZ01/ENTRA/00042</t>
+  </si>
+  <si>
+    <t>00059</t>
+  </si>
+  <si>
+    <t>C-C/00038</t>
   </si>
 </sst>
 </file>
@@ -695,7 +731,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="30.7109375" customWidth="1"/>
@@ -732,7 +768,7 @@
         <v>8</v>
       </c>
       <c r="B2" s="3">
-        <v>45947.40354166667</v>
+        <v>45947.40349537037</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>9</v>
@@ -747,7 +783,7 @@
         <v>11</v>
       </c>
       <c r="G2" s="5">
-        <v>1353.99</v>
+        <v>1314.06</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>12</v>
@@ -758,7 +794,7 @@
         <v>13</v>
       </c>
       <c r="B3" s="3">
-        <v>45947.40657407408</v>
+        <v>45947.40592592592</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>14</v>
@@ -773,7 +809,7 @@
         <v>16</v>
       </c>
       <c r="G3" s="5">
-        <v>1067.22</v>
+        <v>1130.14</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>12</v>
@@ -784,7 +820,7 @@
         <v>17</v>
       </c>
       <c r="B4" s="3">
-        <v>45952.40754629629</v>
+        <v>45952.53523148148</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>18</v>
@@ -799,7 +835,7 @@
         <v>19</v>
       </c>
       <c r="G4" s="5">
-        <v>3748.58</v>
+        <v>3714.7</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>12</v>
@@ -810,22 +846,22 @@
         <v>20</v>
       </c>
       <c r="B5" s="3">
-        <v>45952.40959490741</v>
+        <v>45952.53799768518</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D5" s="4">
         <v>45952</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G5" s="5">
-        <v>4239.84</v>
+        <v>3714.7</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>12</v>
@@ -833,25 +869,25 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B6" s="3">
-        <v>45959.39005787037</v>
+        <v>45952.5390162037</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D6" s="4">
-        <v>45959</v>
+        <v>45952</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="G6" s="5">
-        <v>3303.3</v>
+        <v>4319.7</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>12</v>
@@ -859,10 +895,10 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B7" s="3">
-        <v>45959.39197916666</v>
+        <v>45959.39460648148</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>24</v>
@@ -871,13 +907,13 @@
         <v>45959</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G7" s="5">
-        <v>3873.21</v>
+        <v>3780.04</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>12</v>
@@ -885,25 +921,25 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="3">
+        <v>45959.39613425926</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="4">
+        <v>45959</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="3">
-        <v>45966.38633101852</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" s="4">
-        <v>45966</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>30</v>
-      </c>
       <c r="G8" s="5">
-        <v>4242.26</v>
+        <v>4126.1</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>12</v>
@@ -911,25 +947,25 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B9" s="3">
-        <v>45966.38871527778</v>
+        <v>45966.39165509259</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D9" s="4">
         <v>45966</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G9" s="5">
-        <v>5150.97</v>
+        <v>3523.52</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>12</v>
@@ -937,25 +973,25 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B10" s="3">
-        <v>45973.38270833333</v>
+        <v>45966.39399305556</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D10" s="4">
-        <v>45973</v>
+        <v>45966</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G10" s="5">
-        <v>3564.66</v>
+        <v>4467.32</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>12</v>
@@ -963,10 +999,10 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B11" s="3">
-        <v>45973.38444444445</v>
+        <v>45973.37914351852</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>35</v>
@@ -978,10 +1014,10 @@
         <v>10</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G11" s="5">
-        <v>4773.45</v>
+        <v>4481.84</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>12</v>
@@ -989,25 +1025,25 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="3">
+        <v>45973.38052083334</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="4">
+        <v>45973</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B12" s="3">
-        <v>45980.39841435185</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D12" s="4">
-        <v>45980</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>41</v>
-      </c>
       <c r="G12" s="5">
-        <v>3310.56</v>
+        <v>4038.98</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>12</v>
@@ -1015,13 +1051,13 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B13" s="3">
-        <v>45980.40009259259</v>
+        <v>45980.38145833334</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D13" s="4">
         <v>45980</v>
@@ -1030,10 +1066,10 @@
         <v>10</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G13" s="5">
-        <v>3767.94</v>
+        <v>3574.34</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>12</v>
@@ -1041,25 +1077,25 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B14" s="3">
-        <v>45987.39813657408</v>
+        <v>45980.38202546296</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="D14" s="4">
-        <v>45987</v>
+        <v>45980</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="G14" s="5">
-        <v>3859.9</v>
+        <v>3518.68</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>12</v>
@@ -1067,10 +1103,10 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B15" s="3">
-        <v>45987.39975694445</v>
+        <v>45987.38065972222</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>46</v>
@@ -1082,10 +1118,10 @@
         <v>10</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G15" s="5">
-        <v>4265.25</v>
+        <v>3947.02</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>12</v>
@@ -1093,25 +1129,25 @@
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B16" s="3">
+        <v>45987.38152777778</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16" s="4">
+        <v>45987</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B16" s="3">
-        <v>45994.38989583333</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D16" s="4">
-        <v>45994</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>52</v>
-      </c>
       <c r="G16" s="5">
-        <v>3576.76</v>
+        <v>3695.34</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>12</v>
@@ -1119,13 +1155,13 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B17" s="3">
-        <v>45994.39055555555</v>
+        <v>45995.36248842593</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D17" s="4">
         <v>45994</v>
@@ -1134,10 +1170,10 @@
         <v>10</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G17" s="5">
-        <v>4345.11</v>
+        <v>4157.56</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>12</v>
@@ -1145,25 +1181,25 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B18" s="3">
-        <v>46001.38744212963</v>
+        <v>45995.3641087963</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="D18" s="4">
-        <v>46001</v>
+        <v>45994</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G18" s="5">
-        <v>3492.06</v>
+        <v>3605.8</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>12</v>
@@ -1171,51 +1207,49 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B19" s="3">
-        <v>46001.38807870371</v>
+        <v>46002.33601851852</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D19" s="4">
         <v>46001</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="G19" s="5">
-        <v>4189.02</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="G19" s="2"/>
       <c r="H19" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B20" s="3">
-        <v>46009.35645833334</v>
+        <v>46002.33883101852</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D20" s="4">
-        <v>46009</v>
+        <v>46001</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="G20" s="5">
-        <v>3373.48</v>
+        <v>4414.08</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>12</v>
@@ -1223,25 +1257,25 @@
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B21" s="3">
-        <v>46009.35783564814</v>
+        <v>46002.34972222222</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="D21" s="4">
-        <v>46009</v>
+        <v>46001</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G21" s="5">
-        <v>3767.94</v>
+        <v>3780.04</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>12</v>
@@ -1249,25 +1283,25 @@
     </row>
     <row r="22" spans="1:8">
       <c r="A22" s="2" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B22" s="3">
-        <v>46015.47129629629</v>
+        <v>46009.34543981482</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D22" s="4">
-        <v>46015</v>
+        <v>46008</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="G22" s="5">
-        <v>162.14</v>
+        <v>3927.66</v>
       </c>
       <c r="H22" s="2" t="s">
         <v>12</v>
@@ -1275,25 +1309,25 @@
     </row>
     <row r="23" spans="1:8">
       <c r="A23" s="2" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B23" s="3">
-        <v>46015.47234953703</v>
+        <v>46009.34717592593</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D23" s="4">
-        <v>46015</v>
+        <v>46008</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G23" s="5">
-        <v>163.35</v>
+        <v>4307.6</v>
       </c>
       <c r="H23" s="2" t="s">
         <v>12</v>
@@ -1301,25 +1335,25 @@
     </row>
     <row r="24" spans="1:8">
       <c r="A24" s="2" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B24" s="3">
-        <v>46030.47358796297</v>
+        <v>46020.40893518519</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D24" s="4">
-        <v>46030</v>
+        <v>46020</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="G24" s="5">
-        <v>3789.72</v>
+        <v>162.14</v>
       </c>
       <c r="H24" s="2" t="s">
         <v>12</v>
@@ -1327,25 +1361,25 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B25" s="3">
-        <v>46030.47418981481</v>
+        <v>46020.40989583333</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D25" s="4">
-        <v>46030</v>
+        <v>46020</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="G25" s="5">
-        <v>4265.25</v>
+        <v>157.3</v>
       </c>
       <c r="H25" s="2" t="s">
         <v>12</v>
@@ -1353,25 +1387,25 @@
     </row>
     <row r="26" spans="1:8">
       <c r="A26" s="2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B26" s="3">
-        <v>46036.38193287037</v>
+        <v>46031.37940972222</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D26" s="4">
-        <v>46036</v>
+        <v>46030</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="G26" s="5">
-        <v>3789.72</v>
+        <v>3709.86</v>
       </c>
       <c r="H26" s="2" t="s">
         <v>12</v>
@@ -1379,25 +1413,25 @@
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="2" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B27" s="3">
-        <v>46036.38248842592</v>
+        <v>46031.38127314814</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D27" s="4">
-        <v>46036</v>
+        <v>46030</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="G27" s="5">
-        <v>4105.53</v>
+        <v>4445.54</v>
       </c>
       <c r="H27" s="2" t="s">
         <v>12</v>
@@ -1405,25 +1439,25 @@
     </row>
     <row r="28" spans="1:8">
       <c r="A28" s="2" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B28" s="3">
-        <v>46043.38505787037</v>
+        <v>46036.3792824074</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D28" s="4">
-        <v>46043</v>
+        <v>46036</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="G28" s="5">
-        <v>3869.58</v>
+        <v>3893.78</v>
       </c>
       <c r="H28" s="2" t="s">
         <v>12</v>
@@ -1431,25 +1465,25 @@
     </row>
     <row r="29" spans="1:8">
       <c r="A29" s="2" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B29" s="3">
-        <v>46043.38584490741</v>
+        <v>46036.38003472222</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="D29" s="4">
-        <v>46043</v>
+        <v>46036</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G29" s="5">
-        <v>4599.21</v>
+        <v>3748.58</v>
       </c>
       <c r="H29" s="2" t="s">
         <v>12</v>
@@ -1457,25 +1491,25 @@
     </row>
     <row r="30" spans="1:8">
       <c r="A30" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B30" s="3">
-        <v>46050.39680555555</v>
+        <v>46043.49070601852</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D30" s="4">
-        <v>46050</v>
+        <v>46043</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G30" s="5">
-        <v>3734.06</v>
+        <v>3407.36</v>
       </c>
       <c r="H30" s="2" t="s">
         <v>12</v>
@@ -1483,25 +1517,25 @@
     </row>
     <row r="31" spans="1:8">
       <c r="A31" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B31" s="3">
-        <v>46050.39799768518</v>
+        <v>46043.49137731481</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D31" s="4">
-        <v>46050</v>
+        <v>46043</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="G31" s="5">
-        <v>4548.39</v>
+        <v>4544.76</v>
       </c>
       <c r="H31" s="2" t="s">
         <v>12</v>
@@ -1509,25 +1543,25 @@
     </row>
     <row r="32" spans="1:8">
       <c r="A32" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B32" s="3">
-        <v>46057.42105324074</v>
+        <v>46044.52113425926</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D32" s="4">
-        <v>46057</v>
+        <v>46044</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G32" s="5">
-        <v>7451.18</v>
+        <v>162.14</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>12</v>
@@ -1535,25 +1569,25 @@
     </row>
     <row r="33" spans="1:8">
       <c r="A33" s="2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B33" s="3">
-        <v>46057.42175925926</v>
+        <v>46044.5219212963</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D33" s="4">
-        <v>46057</v>
+        <v>46044</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G33" s="5">
-        <v>8152.98</v>
+        <v>157.3</v>
       </c>
       <c r="H33" s="2" t="s">
         <v>12</v>
@@ -1561,25 +1595,25 @@
     </row>
     <row r="34" spans="1:8">
       <c r="A34" s="2" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B34" s="3">
-        <v>46064.50871527778</v>
+        <v>46051.34006944444</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D34" s="4">
-        <v>46064</v>
+        <v>46050</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G34" s="5">
-        <v>3777.62</v>
+        <v>4038.98</v>
       </c>
       <c r="H34" s="2" t="s">
         <v>12</v>
@@ -1587,27 +1621,157 @@
     </row>
     <row r="35" spans="1:8">
       <c r="A35" s="2" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B35" s="3">
-        <v>46064.50930555556</v>
+        <v>46051.34134259259</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>104</v>
       </c>
       <c r="D35" s="4">
-        <v>46064</v>
+        <v>46050</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F35" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="G35" s="5">
+        <v>4464.9</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B36" s="3">
+        <v>46051.36006944445</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="G35" s="5">
-        <v>4475.79</v>
-      </c>
-      <c r="H35" s="2" t="s">
+      <c r="D36" s="4">
+        <v>46051</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G36" s="5">
+        <v>84.7</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B37" s="3">
+        <v>46057.39192129629</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D37" s="4">
+        <v>46057</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="G37" s="5">
+        <v>6838.92</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B38" s="3">
+        <v>46057.39331018519</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D38" s="4">
+        <v>46057</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="G38" s="5">
+        <v>7545.56</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B39" s="3">
+        <v>46064.37241898148</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D39" s="4">
+        <v>46064</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="G39" s="5">
+        <v>4818.22</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B40" s="3">
+        <v>46064.37310185185</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D40" s="4">
+        <v>46064</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="G40" s="5">
+        <v>4377.78</v>
+      </c>
+      <c r="H40" s="2" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>